<commit_message>
File nhap lieu: them cot 'Ky' cho tung dong — nhieu nguoi cap nhat nhieu thang cung luc
- Tab KY BAO CAO: moi ky mot dong (truoc day ca sheet chi co mot Ma ky)
- Tab DU AN / KHO KHAN / MOC THOI GIAN: them cot 'Ky' o dau, co o chon san
- Script tra ve DANH SACH ky; applyNhapLieu() gop tung ky vao dung ky trung ma
- Kho khan & moc chi thay phan cua nhung du an duoc nhac toi -> Tung them moc
  cho du an cua minh khong lam mat moc cua Thu
</commit_message>
<xml_diff>
--- a/NhapLieu-BaoCaoThang.xlsx
+++ b/NhapLieu-BaoCaoThang.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,14 +51,19 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001B2A5B"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00E03A3C"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00E03A3C"/>
     </font>
     <font>
       <i val="1"/>
       <color rgb="005B6577"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001B2A5B"/>
     </font>
     <font>
       <b val="1"/>
@@ -136,13 +141,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -510,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -537,30 +542,30 @@
       <c r="A4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>1. Tab KỲ BÁO CÁO — sửa mã kỳ, nhãn và ngày chốt số mỗi khi bắt đầu tháng mới.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CỘT 'KỲ' Ở ĐẦU MỖI TAB LÀ QUAN TRỌNG NHẤT:</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. Tab DỰ ÁN — mỗi dự án một dòng: trạng thái, doanh thu, kết quả, kế hoạch.</t>
+          <t>Mỗi dòng tự khai nó thuộc tháng nào, nên hai người có thể cập nhật hai tháng khác nhau</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>3. Tab KHÓ KHĂN — việc cần lãnh đạo hỗ trợ (hiện ngay trang chính của dashboard).</t>
+          <t>cùng lúc — ví dụ Tùng sửa dòng kỳ 2026-08 còn Thư thêm dòng kỳ 2026-07, không ảnh hưởng nhau.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Tab MỐC THỜI GIAN — các mốc go-live, hạn thanh toán, sự kiện trong kỳ.</t>
+          <t>Muốn bổ sung cho tháng khác: chép dòng dự án của mình xuống dưới rồi đổi ô 'Kỳ'.</t>
         </is>
       </c>
     </row>
@@ -568,54 +573,92 @@
       <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>QUY TẮC QUAN TRỌNG:</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1. Tab KỲ BÁO CÁO — mỗi tháng một dòng (nhãn, khoảng thời gian, ngày chốt số).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Cột 'Mã dự án' là khoá nối với dashboard — KHÔNG sửa, không xoá dòng, không đổi thứ tự.</t>
+          <t>2. Tab DỰ ÁN — mỗi dòng = một dự án trong một kỳ: trạng thái, doanh thu, kết quả, kế hoạch.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• Ô nhiều ý: mỗi ý một dòng trong cùng ô (bấm Alt+Enter để xuống dòng). Không đánh số thứ tự.</t>
+          <t>3. Tab KHÓ KHĂN — việc cần lãnh đạo hỗ trợ (hiện ngay trang chính của dashboard).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Doanh thu điền theo ĐƠN VỊ TỶ ĐỒNG, dùng dấu chấm thập phân (ví dụ 2.05 nghĩa là 2,05 tỷ).</t>
+          <t>4. Tab MỐC THỜI GIAN — các mốc go-live, hạn thanh toán, sự kiện trong kỳ.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>• Dòng TripCARE và wBooking: BỎ TRỐNG các cột số — dashboard tự lấy từ Google Sheet doanh thu.</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>• Chưa có số liệu thì để trống, đừng điền số 0 (số 0 sẽ hiển thị là 'đã phát sinh 0 đồng').</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>QUY TẮC QUAN TRỌNG:</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>• Cột 'Mã dự án' là khoá nối với dashboard — KHÔNG sửa. Cột 'Kỳ' chọn từ danh sách có sẵn.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Điền xong không cần làm gì thêm: dashboard tự cập nhật 2 lần/ngày (7h và 17h).</t>
+          <t>• Ô nào để TRỐNG thì dashboard giữ nguyên nội dung cũ, không bị xoá mất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Ô nhiều ý: mỗi ý một dòng trong cùng ô (bấm Alt+Enter để xuống dòng). Không đánh số thứ tự.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>• Doanh thu điền theo ĐƠN VỊ TỶ ĐỒNG, dùng dấu chấm thập phân (ví dụ 2.05 nghĩa là 2,05 tỷ).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>• Dòng TripCARE và wBooking: BỎ TRỐNG các cột số — dashboard tự lấy từ Google Sheet doanh thu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>• Chưa có số liệu thì để trống, đừng điền số 0 (số 0 sẽ hiển thị là 'đã phát sinh 0 đồng').</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Điền xong không cần làm gì thêm: dashboard tự cập nhật 4 lần/ngày (8h, 10h, 14h, 16h).</t>
         </is>
       </c>
     </row>
@@ -630,52 +673,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Trường</t>
+          <t>Mã kỳ
+(không sửa định dạng)</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Giá trị</t>
+          <t>Nhãn hiển thị</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Giải thích</t>
+          <t>Khoảng thời gian</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Chốt số đến ngày</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Mục tiêu năm (tỷ)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Lưu ý chung (không bắt buộc)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Mã kỳ</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Định dạng NĂM-THÁNG, ví dụ 2026-10 cho tháng 10</t>
-        </is>
-      </c>
+          <t>Tháng 08/2026</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>01–31/08/2026</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Nhãn hiển thị</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -683,69 +754,40 @@
           <t>Tháng 09/2026</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Tên hiện trên ô chọn kỳ của dashboard</t>
-        </is>
-      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>01–30/09/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Khoảng thời gian</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>01–30/09/2026</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr"/>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Chốt số đến ngày</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Ngày số liệu được chốt</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Mục tiêu năm (tỷ)</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Mục tiêu doanh thu cả năm của Phòng</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Lưu ý chung</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Câu lưu ý hiện kèm bảng doanh thu (để trống nếu không có)</t>
-        </is>
-      </c>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Thêm tháng mới: chép một dòng ở trên rồi sửa lại — mã kỳ theo định dạng NĂM-THÁNG (2026-10, 2026-11…)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -758,79 +800,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
     <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>Kỳ</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
           <t>Mã dự án
 (không sửa)</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Tên dự án</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Phụ trách</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Trạng thái</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>DT tháng
 (tỷ)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Lũy kế
 (tỷ)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>% KPI năm</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Cùng kỳ 2025
 (tỷ)</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Ghi chú (1–2 câu tóm tắt cho lãnh đạo)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Kết quả trong kỳ
 (mỗi ý một dòng)</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Kế hoạch tiếp theo
 (mỗi ý một dòng)</t>
@@ -840,49 +888,58 @@
     <row r="2" ht="58" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
           <t>tripcare</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>TripCARE</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Hằng</t>
         </is>
       </c>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>(tự động)</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n"/>
       <c r="G2" s="10" t="n"/>
       <c r="H2" s="10" t="n"/>
-      <c r="I2" s="6" t="n"/>
+      <c r="I2" s="10" t="n"/>
       <c r="J2" s="6" t="n"/>
       <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
     </row>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
           <t>spa</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>SPA GoSafe</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Hằng</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
@@ -890,24 +947,29 @@
       <c r="I3" s="6" t="n"/>
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
+      <c r="L3" s="6" t="n"/>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
           <t>bamboocare</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>BambooCARE</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Hằng</t>
         </is>
       </c>
-      <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
       <c r="G4" s="6" t="n"/>
@@ -915,53 +977,63 @@
       <c r="I4" s="6" t="n"/>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
+      <c r="L4" s="6" t="n"/>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
           <t>wbooking</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>wBooking (HIO)</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Hằng</t>
         </is>
       </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>(tự động)</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n"/>
       <c r="G5" s="10" t="n"/>
       <c r="H5" s="10" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="I5" s="10" t="n"/>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
+      <c r="L5" s="6" t="n"/>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
           <t>flightdelay</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Flight Delay</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Hằng</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="6" t="n"/>
@@ -969,24 +1041,29 @@
       <c r="I6" s="6" t="n"/>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
+      <c r="L6" s="6" t="n"/>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
           <t>asahi</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Asahi (NPUV + APUV)</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Thư</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
@@ -994,24 +1071,29 @@
       <c r="I7" s="6" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
+      <c r="L7" s="6" t="n"/>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
           <t>mobifone</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>MobiFone (Cổng BH)</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Thư</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
@@ -1019,24 +1101,29 @@
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
+      <c r="L8" s="6" t="n"/>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
           <t>zalopay</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Zalopay (BHRVMH)</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Thư</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
@@ -1044,24 +1131,29 @@
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
           <t>nnx</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>NNX (Trợ cấp nằm viện)</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Thư</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
@@ -1069,24 +1161,29 @@
       <c r="I10" s="6" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
           <t>plus-ew</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Plus &amp; EW Honda</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Tùng</t>
         </is>
       </c>
-      <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
@@ -1094,24 +1191,29 @@
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
     </row>
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
           <t>viettelstore</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Viettel Store</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Tùng</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="n"/>
@@ -1119,24 +1221,29 @@
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
           <t>sungroup</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Sun Group (BH nhúng)</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Tùng</t>
         </is>
       </c>
-      <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="n"/>
@@ -1144,24 +1251,29 @@
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
           <t>khac</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Các dự án khác</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Tùng</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
@@ -1169,11 +1281,15 @@
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Đang tăng trưởng,Sắp go-live,Cần chú ý,Chờ đối tác"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"2026-07,2026-08,2026-09,2026-10,2026-11,2026-12"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1186,53 +1302,182 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>Kỳ</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
           <t>Mức độ</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Dự án</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Khó khăn / vướng mắc</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Đề xuất lãnh đạo hỗ trợ</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1"/>
-    <row r="3" ht="46" customHeight="1"/>
-    <row r="4" ht="46" customHeight="1"/>
-    <row r="5" ht="46" customHeight="1"/>
-    <row r="6" ht="46" customHeight="1"/>
-    <row r="7" ht="46" customHeight="1"/>
-    <row r="8" ht="46" customHeight="1"/>
-    <row r="9" ht="46" customHeight="1"/>
-    <row r="10" ht="46" customHeight="1"/>
-    <row r="11" ht="46" customHeight="1"/>
-    <row r="12" ht="46" customHeight="1"/>
-    <row r="13" ht="46" customHeight="1"/>
+    <row r="2" ht="46" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="A2:A30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"GẤP,Theo dõi"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A2:A60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"2026-07,2026-08,2026-09,2026-10,2026-11,2026-12"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1245,75 +1490,348 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>Kỳ</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
           <t>Ngày / thời điểm</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Dự án</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Nội dung mốc</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Quan trọng?
 (x)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Trạng thái</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1"/>
-    <row r="3" ht="30" customHeight="1"/>
-    <row r="4" ht="30" customHeight="1"/>
-    <row r="5" ht="30" customHeight="1"/>
-    <row r="6" ht="30" customHeight="1"/>
-    <row r="7" ht="30" customHeight="1"/>
-    <row r="8" ht="30" customHeight="1"/>
-    <row r="9" ht="30" customHeight="1"/>
-    <row r="10" ht="30" customHeight="1"/>
-    <row r="11" ht="30" customHeight="1"/>
-    <row r="12" ht="30" customHeight="1"/>
-    <row r="13" ht="30" customHeight="1"/>
-    <row r="14" ht="30" customHeight="1"/>
-    <row r="15" ht="30" customHeight="1"/>
-    <row r="16" ht="30" customHeight="1"/>
-    <row r="17" ht="30" customHeight="1"/>
-    <row r="18" ht="30" customHeight="1"/>
-    <row r="19" ht="30" customHeight="1"/>
-    <row r="20" ht="30" customHeight="1"/>
-    <row r="21" ht="30" customHeight="1"/>
-    <row r="22" ht="30" customHeight="1"/>
-    <row r="23" ht="30" customHeight="1"/>
-    <row r="24" ht="30" customHeight="1"/>
-    <row r="25" ht="30" customHeight="1"/>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="E2:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Hoàn thành,Đã đến hạn,Trượt hạn"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A2:A60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"2026-07,2026-08,2026-09,2026-10,2026-11,2026-12"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Them cot 'Ho tro' va 'Uu tien' vao sheet Du an; doc cot theo TIEU DE
- Script nhan dien cot theo ten tieu de thay vi vi tri co dinh -> Phong them cot
  hoac doi thu tu cot deu khong lam hong gi
- Cot 'Ho tro' (chon nhan su) va 'Uu tien' 1-5 sao: dashboard cap nhat theo
- Dropdown trang thai trong file mau co them 'Dang thuc hien'
</commit_message>
<xml_diff>
--- a/NhapLieu-BaoCaoThang.xlsx
+++ b/NhapLieu-BaoCaoThang.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -620,43 +620,50 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• Ô nào để TRỐNG thì dashboard giữ nguyên nội dung cũ, không bị xoá mất.</t>
+          <t>• Cột 'Hỗ trợ' và 'Ưu tiên' (1–5 sao) sửa được bất cứ lúc nào, dashboard cập nhật theo.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• Ô nhiều ý: mỗi ý một dòng trong cùng ô (bấm Alt+Enter để xuống dòng). Không đánh số thứ tự.</t>
+          <t>• Ô nào để TRỐNG thì dashboard giữ nguyên nội dung cũ, không bị xoá mất.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>• Doanh thu điền theo ĐƠN VỊ TỶ ĐỒNG, dùng dấu chấm thập phân (ví dụ 2.05 nghĩa là 2,05 tỷ).</t>
+          <t>• Ô nhiều ý: mỗi ý một dòng trong cùng ô (bấm Alt+Enter để xuống dòng). Không đánh số thứ tự.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>• Dòng TripCARE và wBooking: BỎ TRỐNG các cột số — dashboard tự lấy từ Google Sheet doanh thu.</t>
+          <t>• Doanh thu điền theo ĐƠN VỊ TỶ ĐỒNG, dùng dấu chấm thập phân (ví dụ 2.05 nghĩa là 2,05 tỷ).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>• Dòng TripCARE và wBooking: BỎ TRỐNG các cột số — dashboard tự lấy từ Google Sheet doanh thu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>• Chưa có số liệu thì để trống, đừng điền số 0 (số 0 sẽ hiển thị là 'đã phát sinh 0 đồng').</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="2" t="inlineStr"/>
-    </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Điền xong không cần làm gì thêm: dashboard tự cập nhật 4 lần/ngày (8h, 10h, 14h, 16h).</t>
         </is>
@@ -800,21 +807,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
-    <col width="52" customWidth="1" min="11" max="11"/>
-    <col width="52" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="52" customWidth="1" min="13" max="13"/>
+    <col width="52" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -841,44 +850,55 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Hỗ trợ</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Ưu tiên
+(1–5 sao)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>Trạng thái</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>DT tháng
 (tỷ)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Lũy kế
 (tỷ)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>% KPI năm</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Cùng kỳ 2025
 (tỷ)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Ghi chú (1–2 câu tóm tắt cho lãnh đạo)</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Kết quả trong kỳ
 (mỗi ý một dòng)</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Kế hoạch tiếp theo
 (mỗi ý một dòng)</t>
@@ -907,17 +927,19 @@
         </is>
       </c>
       <c r="E2" s="6" t="n"/>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>(tự động)</t>
         </is>
       </c>
-      <c r="G2" s="10" t="n"/>
-      <c r="H2" s="10" t="n"/>
       <c r="I2" s="10" t="n"/>
-      <c r="J2" s="6" t="n"/>
-      <c r="K2" s="6" t="n"/>
+      <c r="J2" s="10" t="n"/>
+      <c r="K2" s="10" t="n"/>
       <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
     </row>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
@@ -948,6 +970,8 @@
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6" t="n"/>
+      <c r="M3" s="6" t="n"/>
+      <c r="N3" s="6" t="n"/>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -978,6 +1002,8 @@
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="6" t="n"/>
+      <c r="M4" s="6" t="n"/>
+      <c r="N4" s="6" t="n"/>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -1001,17 +1027,19 @@
         </is>
       </c>
       <c r="E5" s="6" t="n"/>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>(tự động)</t>
         </is>
       </c>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
       <c r="I5" s="10" t="n"/>
-      <c r="J5" s="6" t="n"/>
-      <c r="K5" s="6" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
       <c r="L5" s="6" t="n"/>
+      <c r="M5" s="6" t="n"/>
+      <c r="N5" s="6" t="n"/>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1042,6 +1070,8 @@
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6" t="n"/>
+      <c r="M6" s="6" t="n"/>
+      <c r="N6" s="6" t="n"/>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
@@ -1072,6 +1102,8 @@
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="6" t="n"/>
+      <c r="M7" s="6" t="n"/>
+      <c r="N7" s="6" t="n"/>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1102,6 +1134,8 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6" t="n"/>
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="6" t="n"/>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
@@ -1132,6 +1166,8 @@
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="6" t="n"/>
+      <c r="M9" s="6" t="n"/>
+      <c r="N9" s="6" t="n"/>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -1162,6 +1198,8 @@
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6" t="n"/>
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6" t="n"/>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
@@ -1192,6 +1230,8 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
+      <c r="N11" s="6" t="n"/>
     </row>
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1222,6 +1262,8 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="n"/>
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6" t="n"/>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
@@ -1252,6 +1294,8 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="6" t="n"/>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -1282,11 +1326,19 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="6" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Đang tăng trưởng,Sắp go-live,Cần chú ý,Chờ đối tác"</formula1>
+  <dataValidations count="4">
+    <dataValidation sqref="G2:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Đang tăng trưởng,Đang thực hiện,Sắp go-live,Cần chú ý,Chờ đối tác"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Hằng,Thư,Tùng,Duy"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
     <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2026-07,2026-08,2026-09,2026-10,2026-11,2026-12"</formula1>

</xml_diff>